<commit_message>
pushing working rendition of the database.
</commit_message>
<xml_diff>
--- a/llacie/database/micro_antibiotics_TRP.xlsx
+++ b/llacie/database/micro_antibiotics_TRP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anish/Code/Pak Lab/llacie/llacie/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCB726D-096C-5641-B599-6FDE0D471AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F112D14-FF1B-4C4C-8227-6DAB4404CEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3080" yWindow="760" windowWidth="24660" windowHeight="17080" xr2:uid="{5FF92C89-5F5C-0F4D-9681-072752D9D6F1}"/>
+    <workbookView xWindow="3080" yWindow="760" windowWidth="24660" windowHeight="17020" xr2:uid="{5FF92C89-5F5C-0F4D-9681-072752D9D6F1}"/>
   </bookViews>
   <sheets>
     <sheet name="antibiotic_map" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="745">
   <si>
     <t>fosfomycin</t>
   </si>
@@ -2267,6 +2267,9 @@
   </si>
   <si>
     <t>ticarcillin/clavulanate</t>
+  </si>
+  <si>
+    <t>Phenoxymethylpenicillin</t>
   </si>
 </sst>
 </file>
@@ -4587,6 +4590,9 @@
       <c r="A179" t="s">
         <v>417</v>
       </c>
+      <c r="B179" t="s">
+        <v>744</v>
+      </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" t="s">

</xml_diff>